<commit_message>
Point hq-ssc-equipment-rooms at SSC ontology V03
The script still named QF_SSC_Ontology_ver02.xlsx, which V03 replaced, so
it died on FileNotFoundError before reading a row. Path only - the sheet
is picked by its header, so V03's Sheet1 is found without further change.

V03 is a straight improvement on what the script reports: 148 rows as
before, but 87 need revision rather than 99, and nothing is newly
flagged. The twelve that clear are real upstream corrections, not
suppressed checks - seven rooms that pointed at entity:Level7_Office0367
with no rdfs:label_en now carry named rooms, and five equipment-to-room
disagreements resolve in favour of what the BMS screen said, e.g.
SSC_CCUB0004 B1.023 QTEL -> B-017 MDF-2 and SSC_DXB0009 B1.020 FM
STORAGE -> B-002 HV Room.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01G5ei61eJmqXtuLmQFDtSnt
</commit_message>
<xml_diff>
--- a/projects/hq-ssc-equipment-rooms/HQ_SSC_equipment_rooms.xlsx
+++ b/projects/hq-ssc-equipment-rooms/HQ_SSC_equipment_rooms.xlsx
@@ -694,7 +694,7 @@
       </c>
       <c r="E2" s="5" t="inlineStr">
         <is>
-          <t>entity:SSC_B1_038_SER-2</t>
+          <t>entity:SSC_B-038_Ser-2</t>
         </is>
       </c>
       <c r="F2" s="5" t="inlineStr">
@@ -731,7 +731,7 @@
       </c>
       <c r="E3" s="5" t="inlineStr">
         <is>
-          <t>entity:SSC_B1_038_SER-2</t>
+          <t>entity:SSC_B-038_Ser-2</t>
         </is>
       </c>
       <c r="F3" s="5" t="inlineStr">
@@ -768,7 +768,7 @@
       </c>
       <c r="E4" s="5" t="inlineStr">
         <is>
-          <t>entity:SSC_B1_038_SER-2</t>
+          <t>entity:SSC_B-038_Ser-2</t>
         </is>
       </c>
       <c r="F4" s="5" t="inlineStr">
@@ -805,7 +805,7 @@
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t>entity:SSC_B1_038_SER-2</t>
+          <t>entity:SSC_B-038_Ser-2</t>
         </is>
       </c>
       <c r="F5" s="5" t="inlineStr">
@@ -854,7 +854,7 @@
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>entity:SSC_B1_038_SER-2</t>
+          <t>entity:SSC_B-038_Ser-2</t>
         </is>
       </c>
       <c r="F6" s="5" t="inlineStr">
@@ -903,7 +903,7 @@
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>entity:SSC_B1_038_SER-2</t>
+          <t>entity:SSC_B-038_Ser-2</t>
         </is>
       </c>
       <c r="F7" s="5" t="inlineStr">
@@ -952,7 +952,7 @@
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>entity:SSC_B1_023_Q_TEL</t>
+          <t>entity:SSC_B-023_Q-Tel</t>
         </is>
       </c>
       <c r="F8" s="5" t="inlineStr">
@@ -967,61 +967,53 @@
       <c r="K8" s="6" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" s="7" t="inlineStr">
+      <c r="A9" s="5" t="inlineStr">
         <is>
           <t>SSC</t>
         </is>
       </c>
-      <c r="B9" s="7" t="inlineStr">
+      <c r="B9" s="5" t="inlineStr">
         <is>
           <t>CCU-B-0004</t>
         </is>
       </c>
-      <c r="C9" s="7" t="inlineStr">
+      <c r="C9" s="5" t="inlineStr">
         <is>
           <t>brick:CRAC</t>
         </is>
       </c>
-      <c r="D9" s="7" t="inlineStr">
+      <c r="D9" s="5" t="inlineStr">
         <is>
           <t>entity:SSC_CCUB0004</t>
         </is>
       </c>
-      <c r="E9" s="7" t="inlineStr">
-        <is>
-          <t>entity:SSC_B1_023_Q_TEL</t>
-        </is>
-      </c>
-      <c r="F9" s="7" t="inlineStr">
-        <is>
-          <t>B1.023 QTEL</t>
-        </is>
-      </c>
-      <c r="G9" s="7" t="inlineStr">
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>entity:SSC_B-017_MDF-2</t>
+        </is>
+      </c>
+      <c r="F9" s="5" t="inlineStr">
+        <is>
+          <t>B1.017 MDF-2</t>
+        </is>
+      </c>
+      <c r="G9" s="5" t="inlineStr">
         <is>
           <t>B.017 MDF-2</t>
         </is>
       </c>
-      <c r="H9" s="7" t="inlineStr">
+      <c r="H9" s="5" t="inlineStr">
         <is>
           <t>BF-part1</t>
         </is>
       </c>
-      <c r="I9" s="7" t="inlineStr">
+      <c r="I9" s="5" t="inlineStr">
         <is>
           <t>ok</t>
         </is>
       </c>
-      <c r="J9" s="7" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="K9" s="8" t="inlineStr">
-        <is>
-          <t>the BMS screen puts it in B.017 MDF-2 and the ontology in B1.023 QTEL</t>
-        </is>
-      </c>
+      <c r="J9" s="5" t="inlineStr"/>
+      <c r="K9" s="6" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
@@ -1046,7 +1038,7 @@
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>entity:SSC_B1_023_Q_TEL</t>
+          <t>entity:SSC_B-023_Q-Tel</t>
         </is>
       </c>
       <c r="F10" s="5" t="inlineStr">
@@ -1083,7 +1075,7 @@
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>entity:SSC_B1_023_Q_TEL</t>
+          <t>entity:SSC_B-023_Q-Tel</t>
         </is>
       </c>
       <c r="F11" s="5" t="inlineStr">
@@ -1132,7 +1124,7 @@
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t>entity:SSC_B1_023_Q_TEL</t>
+          <t>entity:SSC_B-023_Q-Tel</t>
         </is>
       </c>
       <c r="F12" s="5" t="inlineStr">
@@ -1181,7 +1173,7 @@
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t>entity:SSC_B1_023_Q_TEL</t>
+          <t>entity:SSC_B-023_Q-Tel</t>
         </is>
       </c>
       <c r="F13" s="5" t="inlineStr">
@@ -1208,61 +1200,53 @@
       <c r="K13" s="6" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" s="7" t="inlineStr">
+      <c r="A14" s="5" t="inlineStr">
         <is>
           <t>SSC</t>
         </is>
       </c>
-      <c r="B14" s="7" t="inlineStr">
+      <c r="B14" s="5" t="inlineStr">
         <is>
           <t>CCU-B-0007</t>
         </is>
       </c>
-      <c r="C14" s="7" t="inlineStr">
+      <c r="C14" s="5" t="inlineStr">
         <is>
           <t>brick:CRAC</t>
         </is>
       </c>
-      <c r="D14" s="7" t="inlineStr">
+      <c r="D14" s="5" t="inlineStr">
         <is>
           <t>entity:SSC_CCUB0007</t>
         </is>
       </c>
-      <c r="E14" s="7" t="inlineStr">
-        <is>
-          <t>entity:SSC_B1_017_MDF-2</t>
-        </is>
-      </c>
-      <c r="F14" s="7" t="inlineStr">
-        <is>
-          <t>B1.017 MDF-2</t>
-        </is>
-      </c>
-      <c r="G14" s="7" t="inlineStr">
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>entity:SSC_B-026_MDF-Ser-1</t>
+        </is>
+      </c>
+      <c r="F14" s="5" t="inlineStr">
+        <is>
+          <t>B1.026 MDF/SER-1</t>
+        </is>
+      </c>
+      <c r="G14" s="5" t="inlineStr">
         <is>
           <t>B.026 MDF/SER.1</t>
         </is>
       </c>
-      <c r="H14" s="7" t="inlineStr">
+      <c r="H14" s="5" t="inlineStr">
         <is>
           <t>BF-part1</t>
         </is>
       </c>
-      <c r="I14" s="7" t="inlineStr">
+      <c r="I14" s="5" t="inlineStr">
         <is>
           <t>ok</t>
         </is>
       </c>
-      <c r="J14" s="7" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="K14" s="8" t="inlineStr">
-        <is>
-          <t>the BMS screen puts it in B.026 MDF/SER.1 and the ontology in B1.017 MDF-2</t>
-        </is>
-      </c>
+      <c r="J14" s="5" t="inlineStr"/>
+      <c r="K14" s="6" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
@@ -1287,7 +1271,7 @@
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t>entity:SSC_B1_017_MDF-2</t>
+          <t>entity:SSC_B-017_MDF-2</t>
         </is>
       </c>
       <c r="F15" s="5" t="inlineStr">
@@ -1324,7 +1308,7 @@
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t>entity:SSC_B1_014_VENT_PLANT</t>
+          <t>entity:SSC_B-014_Vent-Plant</t>
         </is>
       </c>
       <c r="F16" s="5" t="inlineStr">
@@ -1361,7 +1345,7 @@
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t>entity:SSC_B1_014_VENT_PLANT</t>
+          <t>entity:SSC_B-014_Vent-Plant</t>
         </is>
       </c>
       <c r="F17" s="5" t="inlineStr">
@@ -1398,7 +1382,7 @@
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t>entity:SSC_B1_014_VENT_PLANT</t>
+          <t>entity:SSC_B-014_Vent-Plant</t>
         </is>
       </c>
       <c r="F18" s="5" t="inlineStr">
@@ -1435,7 +1419,7 @@
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t>entity:SSC_B1_014_VENT_PLANT</t>
+          <t>entity:SSC_B-014_Vent-Plant</t>
         </is>
       </c>
       <c r="F19" s="5" t="inlineStr">
@@ -1450,315 +1434,287 @@
       <c r="K19" s="6" t="inlineStr"/>
     </row>
     <row r="20">
-      <c r="A20" s="7" t="inlineStr">
+      <c r="A20" s="5" t="inlineStr">
         <is>
           <t>SSC</t>
         </is>
       </c>
-      <c r="B20" s="7" t="inlineStr">
+      <c r="B20" s="5" t="inlineStr">
         <is>
           <t>GEFB0001</t>
         </is>
       </c>
-      <c r="C20" s="7" t="inlineStr">
+      <c r="C20" s="5" t="inlineStr">
         <is>
           <t>brick:Exhaust_Fan</t>
         </is>
       </c>
-      <c r="D20" s="7" t="inlineStr">
+      <c r="D20" s="5" t="inlineStr">
         <is>
           <t>entity:SSC_GEFB0001</t>
         </is>
       </c>
-      <c r="E20" s="7" t="inlineStr">
-        <is>
-          <t>entity:Level7_Office0367</t>
-        </is>
-      </c>
-      <c r="F20" s="7" t="inlineStr"/>
-      <c r="G20" s="7" t="inlineStr"/>
-      <c r="H20" s="7" t="inlineStr"/>
-      <c r="I20" s="7" t="inlineStr"/>
-      <c r="J20" s="7" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="K20" s="8" t="inlineStr">
-        <is>
-          <t>the room entity entity:Level7_Office0367 carries no rdfs:label_en, so it has no readable name</t>
-        </is>
-      </c>
+      <c r="E20" s="5" t="inlineStr">
+        <is>
+          <t>entity:SSC_B-008_Vent-Plant</t>
+        </is>
+      </c>
+      <c r="F20" s="5" t="inlineStr">
+        <is>
+          <t>B1.008 VENT PLANT</t>
+        </is>
+      </c>
+      <c r="G20" s="5" t="inlineStr"/>
+      <c r="H20" s="5" t="inlineStr"/>
+      <c r="I20" s="5" t="inlineStr"/>
+      <c r="J20" s="5" t="inlineStr"/>
+      <c r="K20" s="6" t="inlineStr"/>
     </row>
     <row r="21">
-      <c r="A21" s="7" t="inlineStr">
+      <c r="A21" s="5" t="inlineStr">
         <is>
           <t>SSC</t>
         </is>
       </c>
-      <c r="B21" s="7" t="inlineStr">
+      <c r="B21" s="5" t="inlineStr">
         <is>
           <t>KEF-1F-0103</t>
         </is>
       </c>
-      <c r="C21" s="7" t="inlineStr">
+      <c r="C21" s="5" t="inlineStr">
         <is>
           <t>brick:Exhaust_Fan</t>
         </is>
       </c>
-      <c r="D21" s="7" t="inlineStr">
+      <c r="D21" s="5" t="inlineStr">
         <is>
           <t>entity:SSC_KEF0103</t>
         </is>
       </c>
-      <c r="E21" s="7" t="inlineStr">
-        <is>
-          <t>entity:Level7_Office0367</t>
-        </is>
-      </c>
-      <c r="F21" s="7" t="inlineStr"/>
-      <c r="G21" s="7" t="inlineStr">
+      <c r="E21" s="5" t="inlineStr">
+        <is>
+          <t>entity:SSC_01-005_Kitchen</t>
+        </is>
+      </c>
+      <c r="F21" s="5" t="inlineStr">
+        <is>
+          <t>1.005 KITCHEN</t>
+        </is>
+      </c>
+      <c r="G21" s="5" t="inlineStr">
         <is>
           <t>01.005 KITCHEN</t>
         </is>
       </c>
-      <c r="H21" s="7" t="inlineStr">
+      <c r="H21" s="5" t="inlineStr">
         <is>
           <t>FF-part2</t>
         </is>
       </c>
-      <c r="I21" s="7" t="inlineStr">
+      <c r="I21" s="5" t="inlineStr">
         <is>
           <t>ok</t>
         </is>
       </c>
-      <c r="J21" s="7" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="K21" s="8" t="inlineStr">
-        <is>
-          <t>the room entity entity:Level7_Office0367 carries no rdfs:label_en, so it has no readable name; the BMS screen puts it in 01.005 KITCHEN and the ontology in entity:Level7_Office0367</t>
-        </is>
-      </c>
+      <c r="J21" s="5" t="inlineStr"/>
+      <c r="K21" s="6" t="inlineStr"/>
     </row>
     <row r="22">
-      <c r="A22" s="7" t="inlineStr">
+      <c r="A22" s="5" t="inlineStr">
         <is>
           <t>SSC</t>
         </is>
       </c>
-      <c r="B22" s="7" t="inlineStr">
+      <c r="B22" s="5" t="inlineStr">
         <is>
           <t>KEF0303</t>
         </is>
       </c>
-      <c r="C22" s="7" t="inlineStr">
+      <c r="C22" s="5" t="inlineStr">
         <is>
           <t>brick:Exhaust_Fan</t>
         </is>
       </c>
-      <c r="D22" s="7" t="inlineStr">
+      <c r="D22" s="5" t="inlineStr">
         <is>
           <t>entity:SSC_KEF0303</t>
         </is>
       </c>
-      <c r="E22" s="7" t="inlineStr">
-        <is>
-          <t>entity:Level7_Office0367</t>
-        </is>
-      </c>
-      <c r="F22" s="7" t="inlineStr"/>
-      <c r="G22" s="7" t="inlineStr"/>
-      <c r="H22" s="7" t="inlineStr"/>
-      <c r="I22" s="7" t="inlineStr"/>
-      <c r="J22" s="7" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="K22" s="8" t="inlineStr">
-        <is>
-          <t>the room entity entity:Level7_Office0367 carries no rdfs:label_en, so it has no readable name</t>
-        </is>
-      </c>
+      <c r="E22" s="5" t="inlineStr">
+        <is>
+          <t>entity:SSC_03-049_IT-Office</t>
+        </is>
+      </c>
+      <c r="F22" s="5" t="inlineStr">
+        <is>
+          <t>3.049 IT OFFICE</t>
+        </is>
+      </c>
+      <c r="G22" s="5" t="inlineStr"/>
+      <c r="H22" s="5" t="inlineStr"/>
+      <c r="I22" s="5" t="inlineStr"/>
+      <c r="J22" s="5" t="inlineStr"/>
+      <c r="K22" s="6" t="inlineStr"/>
     </row>
     <row r="23">
-      <c r="A23" s="7" t="inlineStr">
+      <c r="A23" s="5" t="inlineStr">
         <is>
           <t>SSC</t>
         </is>
       </c>
-      <c r="B23" s="7" t="inlineStr">
+      <c r="B23" s="5" t="inlineStr">
         <is>
           <t>TEF-1F-0101</t>
         </is>
       </c>
-      <c r="C23" s="7" t="inlineStr">
+      <c r="C23" s="5" t="inlineStr">
         <is>
           <t>brick:Exhaust_Fan</t>
         </is>
       </c>
-      <c r="D23" s="7" t="inlineStr">
+      <c r="D23" s="5" t="inlineStr">
         <is>
           <t>entity:SSC_TEF0101</t>
         </is>
       </c>
-      <c r="E23" s="7" t="inlineStr">
-        <is>
-          <t>entity:Level7_Office0367</t>
-        </is>
-      </c>
-      <c r="F23" s="7" t="inlineStr"/>
-      <c r="G23" s="7" t="inlineStr">
+      <c r="E23" s="5" t="inlineStr">
+        <is>
+          <t>entity:SSC_01-028_Corridor</t>
+        </is>
+      </c>
+      <c r="F23" s="5" t="inlineStr">
+        <is>
+          <t>1.028 CORRIDOR</t>
+        </is>
+      </c>
+      <c r="G23" s="5" t="inlineStr">
         <is>
           <t>01.028 CORRIDOR</t>
         </is>
       </c>
-      <c r="H23" s="7" t="inlineStr">
+      <c r="H23" s="5" t="inlineStr">
         <is>
           <t>FF-part2</t>
         </is>
       </c>
-      <c r="I23" s="7" t="inlineStr">
+      <c r="I23" s="5" t="inlineStr">
         <is>
           <t>ok</t>
         </is>
       </c>
-      <c r="J23" s="7" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="K23" s="8" t="inlineStr">
-        <is>
-          <t>the room entity entity:Level7_Office0367 carries no rdfs:label_en, so it has no readable name; the BMS screen puts it in 01.028 CORRIDOR and the ontology in entity:Level7_Office0367</t>
-        </is>
-      </c>
+      <c r="J23" s="5" t="inlineStr"/>
+      <c r="K23" s="6" t="inlineStr"/>
     </row>
     <row r="24">
-      <c r="A24" s="7" t="inlineStr">
+      <c r="A24" s="5" t="inlineStr">
         <is>
           <t>SSC</t>
         </is>
       </c>
-      <c r="B24" s="7" t="inlineStr">
+      <c r="B24" s="5" t="inlineStr">
         <is>
           <t>TEF0102</t>
         </is>
       </c>
-      <c r="C24" s="7" t="inlineStr">
+      <c r="C24" s="5" t="inlineStr">
         <is>
           <t>brick:Exhaust_Fan</t>
         </is>
       </c>
-      <c r="D24" s="7" t="inlineStr">
+      <c r="D24" s="5" t="inlineStr">
         <is>
           <t>entity:SSC_TEF0102</t>
         </is>
       </c>
-      <c r="E24" s="7" t="inlineStr">
-        <is>
-          <t>entity:Level7_Office0367</t>
-        </is>
-      </c>
-      <c r="F24" s="7" t="inlineStr"/>
-      <c r="G24" s="7" t="inlineStr"/>
-      <c r="H24" s="7" t="inlineStr"/>
-      <c r="I24" s="7" t="inlineStr"/>
-      <c r="J24" s="7" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="K24" s="8" t="inlineStr">
-        <is>
-          <t>the room entity entity:Level7_Office0367 carries no rdfs:label_en, so it has no readable name</t>
-        </is>
-      </c>
+      <c r="E24" s="5" t="inlineStr">
+        <is>
+          <t>entity:SSC_01-206_Corridor</t>
+        </is>
+      </c>
+      <c r="F24" s="5" t="inlineStr">
+        <is>
+          <t>1.206 CORRIDOR</t>
+        </is>
+      </c>
+      <c r="G24" s="5" t="inlineStr"/>
+      <c r="H24" s="5" t="inlineStr"/>
+      <c r="I24" s="5" t="inlineStr"/>
+      <c r="J24" s="5" t="inlineStr"/>
+      <c r="K24" s="6" t="inlineStr"/>
     </row>
     <row r="25">
-      <c r="A25" s="7" t="inlineStr">
+      <c r="A25" s="5" t="inlineStr">
         <is>
           <t>SSC</t>
         </is>
       </c>
-      <c r="B25" s="7" t="inlineStr">
+      <c r="B25" s="5" t="inlineStr">
         <is>
           <t>TEF0301</t>
         </is>
       </c>
-      <c r="C25" s="7" t="inlineStr">
+      <c r="C25" s="5" t="inlineStr">
         <is>
           <t>brick:Exhaust_Fan</t>
         </is>
       </c>
-      <c r="D25" s="7" t="inlineStr">
+      <c r="D25" s="5" t="inlineStr">
         <is>
           <t>entity:SSC_TEF0301</t>
         </is>
       </c>
-      <c r="E25" s="7" t="inlineStr">
-        <is>
-          <t>entity:Level7_Office0367</t>
-        </is>
-      </c>
-      <c r="F25" s="7" t="inlineStr"/>
-      <c r="G25" s="7" t="inlineStr"/>
-      <c r="H25" s="7" t="inlineStr"/>
-      <c r="I25" s="7" t="inlineStr"/>
-      <c r="J25" s="7" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="K25" s="8" t="inlineStr">
-        <is>
-          <t>the room entity entity:Level7_Office0367 carries no rdfs:label_en, so it has no readable name</t>
-        </is>
-      </c>
+      <c r="E25" s="5" t="inlineStr">
+        <is>
+          <t>entity:SSC_03-038_Server-Room</t>
+        </is>
+      </c>
+      <c r="F25" s="5" t="inlineStr">
+        <is>
+          <t>3.038 IT SERVER ROOM</t>
+        </is>
+      </c>
+      <c r="G25" s="5" t="inlineStr"/>
+      <c r="H25" s="5" t="inlineStr"/>
+      <c r="I25" s="5" t="inlineStr"/>
+      <c r="J25" s="5" t="inlineStr"/>
+      <c r="K25" s="6" t="inlineStr"/>
     </row>
     <row r="26">
-      <c r="A26" s="7" t="inlineStr">
+      <c r="A26" s="5" t="inlineStr">
         <is>
           <t>SSC</t>
         </is>
       </c>
-      <c r="B26" s="7" t="inlineStr">
+      <c r="B26" s="5" t="inlineStr">
         <is>
           <t>TEF0302</t>
         </is>
       </c>
-      <c r="C26" s="7" t="inlineStr">
+      <c r="C26" s="5" t="inlineStr">
         <is>
           <t>brick:Exhaust_Fan</t>
         </is>
       </c>
-      <c r="D26" s="7" t="inlineStr">
+      <c r="D26" s="5" t="inlineStr">
         <is>
           <t>entity:SSC_TEF0302</t>
         </is>
       </c>
-      <c r="E26" s="7" t="inlineStr">
-        <is>
-          <t>entity:Level7_Office0367</t>
-        </is>
-      </c>
-      <c r="F26" s="7" t="inlineStr"/>
-      <c r="G26" s="7" t="inlineStr"/>
-      <c r="H26" s="7" t="inlineStr"/>
-      <c r="I26" s="7" t="inlineStr"/>
-      <c r="J26" s="7" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="K26" s="8" t="inlineStr">
-        <is>
-          <t>the room entity entity:Level7_Office0367 carries no rdfs:label_en, so it has no readable name</t>
-        </is>
-      </c>
+      <c r="E26" s="5" t="inlineStr">
+        <is>
+          <t>entity:SSC_03-045_Janitors-Closet</t>
+        </is>
+      </c>
+      <c r="F26" s="5" t="inlineStr">
+        <is>
+          <t>3.045 JANITOR'S CLOSET</t>
+        </is>
+      </c>
+      <c r="G26" s="5" t="inlineStr"/>
+      <c r="H26" s="5" t="inlineStr"/>
+      <c r="I26" s="5" t="inlineStr"/>
+      <c r="J26" s="5" t="inlineStr"/>
+      <c r="K26" s="6" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="5" t="inlineStr">
@@ -1783,7 +1739,7 @@
       </c>
       <c r="E27" s="5" t="inlineStr">
         <is>
-          <t>entity:SSC_B1_014_VENT_PLANT</t>
+          <t>entity:SSC_B-014_Vent-Plant</t>
         </is>
       </c>
       <c r="F27" s="5" t="inlineStr">
@@ -1820,7 +1776,7 @@
       </c>
       <c r="E28" s="5" t="inlineStr">
         <is>
-          <t>entity:SSC_B1_014_VENT_PLANT</t>
+          <t>entity:SSC_B-014_Vent-Plant</t>
         </is>
       </c>
       <c r="F28" s="5" t="inlineStr">
@@ -1857,7 +1813,7 @@
       </c>
       <c r="E29" s="5" t="inlineStr">
         <is>
-          <t>entity:SSC_B1_014_VENT_PLANT</t>
+          <t>entity:SSC_B-014_Vent-Plant</t>
         </is>
       </c>
       <c r="F29" s="5" t="inlineStr">
@@ -1894,7 +1850,7 @@
       </c>
       <c r="E30" s="5" t="inlineStr">
         <is>
-          <t>entity:SSC_B1_014_VENT_PLANT</t>
+          <t>entity:SSC_B-014_Vent-Plant</t>
         </is>
       </c>
       <c r="F30" s="5" t="inlineStr">
@@ -1931,7 +1887,7 @@
       </c>
       <c r="E31" s="5" t="inlineStr">
         <is>
-          <t>entity:SSC_B1_014_VENT_PLANT</t>
+          <t>entity:SSC_B-014_Vent-Plant</t>
         </is>
       </c>
       <c r="F31" s="5" t="inlineStr">
@@ -1946,118 +1902,102 @@
       <c r="K31" s="6" t="inlineStr"/>
     </row>
     <row r="32">
-      <c r="A32" s="7" t="inlineStr">
+      <c r="A32" s="5" t="inlineStr">
         <is>
           <t>SSC</t>
         </is>
       </c>
-      <c r="B32" s="7" t="inlineStr">
+      <c r="B32" s="5" t="inlineStr">
         <is>
           <t>DX-B-0001</t>
         </is>
       </c>
-      <c r="C32" s="7" t="inlineStr">
+      <c r="C32" s="5" t="inlineStr">
         <is>
           <t>para:DXUnit</t>
         </is>
       </c>
-      <c r="D32" s="7" t="inlineStr">
+      <c r="D32" s="5" t="inlineStr">
         <is>
           <t>entity:SSC_DXB0001</t>
         </is>
       </c>
-      <c r="E32" s="7" t="inlineStr">
-        <is>
-          <t>entity:SSC_B1_005_UPS</t>
-        </is>
-      </c>
-      <c r="F32" s="7" t="inlineStr">
-        <is>
-          <t>B1.005 UPS</t>
-        </is>
-      </c>
-      <c r="G32" s="7" t="inlineStr">
+      <c r="E32" s="5" t="inlineStr">
+        <is>
+          <t>entity:SSC_B-022_Ssp</t>
+        </is>
+      </c>
+      <c r="F32" s="5" t="inlineStr">
+        <is>
+          <t>B1.022 SSP</t>
+        </is>
+      </c>
+      <c r="G32" s="5" t="inlineStr">
         <is>
           <t>B.022 SSP</t>
         </is>
       </c>
-      <c r="H32" s="7" t="inlineStr">
+      <c r="H32" s="5" t="inlineStr">
         <is>
           <t>BF-part1</t>
         </is>
       </c>
-      <c r="I32" s="7" t="inlineStr">
+      <c r="I32" s="5" t="inlineStr">
         <is>
           <t>check</t>
         </is>
       </c>
-      <c r="J32" s="7" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="K32" s="8" t="inlineStr">
-        <is>
-          <t>the BMS screen puts it in B.022 SSP and the ontology in B1.005 UPS; and the screen reading was itself marked as wanting a second look when it was made</t>
-        </is>
-      </c>
+      <c r="J32" s="5" t="inlineStr"/>
+      <c r="K32" s="6" t="inlineStr"/>
     </row>
     <row r="33">
-      <c r="A33" s="7" t="inlineStr">
+      <c r="A33" s="5" t="inlineStr">
         <is>
           <t>SSC</t>
         </is>
       </c>
-      <c r="B33" s="7" t="inlineStr">
+      <c r="B33" s="5" t="inlineStr">
         <is>
           <t>DX-B-0002</t>
         </is>
       </c>
-      <c r="C33" s="7" t="inlineStr">
+      <c r="C33" s="5" t="inlineStr">
         <is>
           <t>para:DXUnit</t>
         </is>
       </c>
-      <c r="D33" s="7" t="inlineStr">
+      <c r="D33" s="5" t="inlineStr">
         <is>
           <t>entity:SSC_DXB0002</t>
         </is>
       </c>
-      <c r="E33" s="7" t="inlineStr">
-        <is>
-          <t>entity:SSC_B1_005_UPS</t>
-        </is>
-      </c>
-      <c r="F33" s="7" t="inlineStr">
-        <is>
-          <t>B1.005 UPS</t>
-        </is>
-      </c>
-      <c r="G33" s="7" t="inlineStr">
+      <c r="E33" s="5" t="inlineStr">
+        <is>
+          <t>entity:SSC_B-022_Ssp</t>
+        </is>
+      </c>
+      <c r="F33" s="5" t="inlineStr">
+        <is>
+          <t>B1.022 SSP</t>
+        </is>
+      </c>
+      <c r="G33" s="5" t="inlineStr">
         <is>
           <t>B.022 SSP</t>
         </is>
       </c>
-      <c r="H33" s="7" t="inlineStr">
+      <c r="H33" s="5" t="inlineStr">
         <is>
           <t>BF-part1</t>
         </is>
       </c>
-      <c r="I33" s="7" t="inlineStr">
+      <c r="I33" s="5" t="inlineStr">
         <is>
           <t>check</t>
         </is>
       </c>
-      <c r="J33" s="7" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="K33" s="8" t="inlineStr">
-        <is>
-          <t>the BMS screen puts it in B.022 SSP and the ontology in B1.005 UPS; and the screen reading was itself marked as wanting a second look when it was made</t>
-        </is>
-      </c>
+      <c r="J33" s="5" t="inlineStr"/>
+      <c r="K33" s="6" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="5" t="inlineStr">
@@ -2082,7 +2022,7 @@
       </c>
       <c r="E34" s="5" t="inlineStr">
         <is>
-          <t>entity:SSC_B1_005_UPS</t>
+          <t>entity:SSC_B-005_UPS</t>
         </is>
       </c>
       <c r="F34" s="5" t="inlineStr">
@@ -2131,7 +2071,7 @@
       </c>
       <c r="E35" s="7" t="inlineStr">
         <is>
-          <t>entity:SSC_B1_005_UPS</t>
+          <t>entity:SSC_B-005_UPS</t>
         </is>
       </c>
       <c r="F35" s="7" t="inlineStr">
@@ -2188,7 +2128,7 @@
       </c>
       <c r="E36" s="5" t="inlineStr">
         <is>
-          <t>entity:SSC_B1_004_MV_SWITCH_ROOM</t>
+          <t>entity:SSC_B-004_MV-Switch-Room</t>
         </is>
       </c>
       <c r="F36" s="5" t="inlineStr">
@@ -2225,12 +2165,12 @@
       </c>
       <c r="E37" s="7" t="inlineStr">
         <is>
-          <t>entity:SSC_B1_004_MV_SWITCH_ROOM</t>
+          <t>entity:SSC_B-033_Closet</t>
         </is>
       </c>
       <c r="F37" s="7" t="inlineStr">
         <is>
-          <t>B1.004 MV SWITCH ROOM</t>
+          <t>B.033 CLOSET</t>
         </is>
       </c>
       <c r="G37" s="7" t="inlineStr">
@@ -2255,7 +2195,7 @@
       </c>
       <c r="K37" s="8" t="inlineStr">
         <is>
-          <t>the BMS screen puts it in B.001 FM STORAGE and the ontology in B1.004 MV SWITCH ROOM</t>
+          <t>the BMS screen puts it in B.001 FM STORAGE and the ontology in B.033 CLOSET</t>
         </is>
       </c>
     </row>
@@ -2282,12 +2222,12 @@
       </c>
       <c r="E38" s="7" t="inlineStr">
         <is>
-          <t>entity:SSC_B1_019_FM_STORAGE</t>
+          <t>entity:SSC_B-003_Transformer</t>
         </is>
       </c>
       <c r="F38" s="7" t="inlineStr">
         <is>
-          <t>B1.019 FM STORAGE</t>
+          <t>B1.003 TRANSFORMER</t>
         </is>
       </c>
       <c r="G38" s="7" t="inlineStr">
@@ -2312,7 +2252,7 @@
       </c>
       <c r="K38" s="8" t="inlineStr">
         <is>
-          <t>the BMS screen puts it in B.006 SERVICE AREA and the ontology in B1.019 FM STORAGE</t>
+          <t>the BMS screen puts it in B.006 SERVICE AREA and the ontology in B1.003 TRANSFORMER</t>
         </is>
       </c>
     </row>
@@ -2339,12 +2279,12 @@
       </c>
       <c r="E39" s="7" t="inlineStr">
         <is>
-          <t>entity:SSC_B1_019_FM_STORAGE</t>
+          <t>entity:SSC_B-003_Transformer</t>
         </is>
       </c>
       <c r="F39" s="7" t="inlineStr">
         <is>
-          <t>B1.019 FM STORAGE</t>
+          <t>B1.003 TRANSFORMER</t>
         </is>
       </c>
       <c r="G39" s="7" t="inlineStr">
@@ -2369,66 +2309,58 @@
       </c>
       <c r="K39" s="8" t="inlineStr">
         <is>
-          <t>the BMS screen puts it in B.008 VENT PLANT and the ontology in B1.019 FM STORAGE</t>
+          <t>the BMS screen puts it in B.008 VENT PLANT and the ontology in B1.003 TRANSFORMER</t>
         </is>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="7" t="inlineStr">
+      <c r="A40" s="5" t="inlineStr">
         <is>
           <t>SSC</t>
         </is>
       </c>
-      <c r="B40" s="7" t="inlineStr">
+      <c r="B40" s="5" t="inlineStr">
         <is>
           <t>DX-B-0009</t>
         </is>
       </c>
-      <c r="C40" s="7" t="inlineStr">
+      <c r="C40" s="5" t="inlineStr">
         <is>
           <t>para:DXUnit</t>
         </is>
       </c>
-      <c r="D40" s="7" t="inlineStr">
+      <c r="D40" s="5" t="inlineStr">
         <is>
           <t>entity:SSC_DXB0009</t>
         </is>
       </c>
-      <c r="E40" s="7" t="inlineStr">
-        <is>
-          <t>entity:SSC_B1_020_FM_STORAGE</t>
-        </is>
-      </c>
-      <c r="F40" s="7" t="inlineStr">
-        <is>
-          <t>B1.020 FM STORAGE</t>
-        </is>
-      </c>
-      <c r="G40" s="7" t="inlineStr">
+      <c r="E40" s="5" t="inlineStr">
+        <is>
+          <t>entity:SSC_B-002_HV-Room</t>
+        </is>
+      </c>
+      <c r="F40" s="5" t="inlineStr">
+        <is>
+          <t>B1.002 HV</t>
+        </is>
+      </c>
+      <c r="G40" s="5" t="inlineStr">
         <is>
           <t>B.002 HV ROOM</t>
         </is>
       </c>
-      <c r="H40" s="7" t="inlineStr">
+      <c r="H40" s="5" t="inlineStr">
         <is>
           <t>BF-part2</t>
         </is>
       </c>
-      <c r="I40" s="7" t="inlineStr">
+      <c r="I40" s="5" t="inlineStr">
         <is>
           <t>ok</t>
         </is>
       </c>
-      <c r="J40" s="7" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="K40" s="8" t="inlineStr">
-        <is>
-          <t>the BMS screen puts it in B.002 HV ROOM and the ontology in B1.020 FM STORAGE</t>
-        </is>
-      </c>
+      <c r="J40" s="5" t="inlineStr"/>
+      <c r="K40" s="6" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="7" t="inlineStr">
@@ -2453,12 +2385,12 @@
       </c>
       <c r="E41" s="7" t="inlineStr">
         <is>
-          <t>entity:SSC_B1_021_FM_STORAGE</t>
+          <t>entity:SSC_B-002_HV-Room</t>
         </is>
       </c>
       <c r="F41" s="7" t="inlineStr">
         <is>
-          <t>B1.021 FM STORAGE</t>
+          <t>B1.002 HV</t>
         </is>
       </c>
       <c r="G41" s="7" t="inlineStr">
@@ -2483,7 +2415,7 @@
       </c>
       <c r="K41" s="8" t="inlineStr">
         <is>
-          <t>the BMS screen puts it in B.033 CLOSET and the ontology in B1.021 FM STORAGE; and the screen reading was itself marked as wanting a second look when it was made</t>
+          <t>the BMS screen puts it in B.033 CLOSET and the ontology in B1.002 HV; and the screen reading was itself marked as wanting a second look when it was made</t>
         </is>
       </c>
     </row>
@@ -2510,7 +2442,7 @@
       </c>
       <c r="E42" s="5" t="inlineStr">
         <is>
-          <t>entity:SSC_B1_012_GENERATOR</t>
+          <t>entity:SSC_B-012_Generator</t>
         </is>
       </c>
       <c r="F42" s="5" t="inlineStr">
@@ -7263,21 +7195,21 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="9" t="inlineStr">
+      <c r="A12" s="10" t="inlineStr">
         <is>
           <t>SSC</t>
         </is>
       </c>
-      <c r="B12" s="9" t="inlineStr">
+      <c r="B12" s="10" t="inlineStr">
         <is>
           <t>brick:CRAC</t>
         </is>
       </c>
-      <c r="C12" s="9" t="n">
+      <c r="C12" s="10" t="n">
         <v>14</v>
       </c>
-      <c r="D12" s="9" t="n">
-        <v>2</v>
+      <c r="D12" s="10" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="13">
@@ -7299,21 +7231,21 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="9" t="inlineStr">
+      <c r="A14" s="10" t="inlineStr">
         <is>
           <t>SSC</t>
         </is>
       </c>
-      <c r="B14" s="9" t="inlineStr">
+      <c r="B14" s="10" t="inlineStr">
         <is>
           <t>brick:Exhaust_Fan</t>
         </is>
       </c>
-      <c r="C14" s="9" t="n">
+      <c r="C14" s="10" t="n">
         <v>7</v>
       </c>
-      <c r="D14" s="9" t="n">
-        <v>7</v>
+      <c r="D14" s="10" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="15">
@@ -7349,7 +7281,7 @@
         <v>10</v>
       </c>
       <c r="D16" s="9" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="17">

</xml_diff>